<commit_message>
feat: add DSUB6X2, PSUB10X2, BLENDSCSUB10 subwoofers
Adds three new subwoofer models to catalog and AVIATOR_BIBLE:
- DSUB6X2: Deep collection, 6Ω lo-z, 90dB sens, 120W program
- PSUB10X2: Pro collection, 4Ω tappable (300/150/75W), 94dB sens, 600W program
- BLENDSCSUB10: BLENDS collection, 4Ω lo-z, 90dB sens, 200W program

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AVIATOR_BIBLE.xlsx
+++ b/AVIATOR_BIBLE.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT150"/>
+  <dimension ref="A1:AT153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12723,6 +12723,192 @@
         </is>
       </c>
     </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Origin Acoustics</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>DSUB6X2</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>each (ea)</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>In-Ceiling</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Subwoofer</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>Indoor</t>
+        </is>
+      </c>
+      <c r="AK151" t="inlineStr">
+        <is>
+          <t>Handling: 60W Pink Noise / 120W Program / 240W Peak</t>
+        </is>
+      </c>
+      <c r="AN151" t="inlineStr">
+        <is>
+          <t>6 Ohm</t>
+        </is>
+      </c>
+      <c r="AO151" t="inlineStr">
+        <is>
+          <t>90dB @ 1m</t>
+        </is>
+      </c>
+      <c r="AR151" t="inlineStr">
+        <is>
+          <t>Three Chamber Bandpass Vibration Canceling, In-Ceiling Subwoofer</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Origin Acoustics</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>PSUB10X2</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>each (ea)</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Surface Mount</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Subwoofer</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>Indoor</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>300W-2000W @ 4Ω</t>
+        </is>
+      </c>
+      <c r="AK152" t="inlineStr">
+        <is>
+          <t>Handling: 300W Pink Noise / 600W Program / 1200W Peak</t>
+        </is>
+      </c>
+      <c r="AN152" t="inlineStr">
+        <is>
+          <t>4 Ohm</t>
+        </is>
+      </c>
+      <c r="AO152" t="inlineStr">
+        <is>
+          <t>94dB (2.83V/1m, Free Space)</t>
+        </is>
+      </c>
+      <c r="AQ152" t="inlineStr">
+        <is>
+          <t>70V: 300W, 150W, 75W</t>
+        </is>
+      </c>
+      <c r="AR152" t="inlineStr">
+        <is>
+          <t>Dual 10" Bandpass Surface Mount Subwoofer</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Origin Acoustics</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>BLENDSCSUB10</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>each (ea)</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>In-Wall</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Subwoofer</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>BLENDS</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Indoor</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>LF-50W to 400W @ 4Ω</t>
+        </is>
+      </c>
+      <c r="AK153" t="inlineStr">
+        <is>
+          <t>Handling: 200W Program / 400W Peak</t>
+        </is>
+      </c>
+      <c r="AN153" t="inlineStr">
+        <is>
+          <t>4 Ohm</t>
+        </is>
+      </c>
+      <c r="AO153" t="inlineStr">
+        <is>
+          <t>90dB @ 1m</t>
+        </is>
+      </c>
+      <c r="AR153" t="inlineStr">
+        <is>
+          <t>Ported In-Wall Subwoofer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>